<commit_message>
Fixed low FG function
</commit_message>
<xml_diff>
--- a/Data/Flaming Gorge DROA Release.xlsx
+++ b/Data/Flaming Gorge DROA Release.xlsx
@@ -5,20 +5,31 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b3dc8a6658ea5b0c/Desktop/Research/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b3dc8a6658ea5b0c/Desktop/Research/LakePowellElev/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_F25DC773A252ABDACC1048FBC9994CD85BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C0FC999-60B8-44F6-8BEB-33062B9C02EE}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="11_F25DC773A252ABDACC1048FBC9994CD85BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FDC638B-898D-4F17-82D2-1479A990234E}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="2388" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -371,7 +382,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D5:F17"/>
+  <dimension ref="D5:I19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="5" spans="4:6" x14ac:dyDescent="0.3">
@@ -390,7 +401,7 @@
         <v>46168</v>
       </c>
       <c r="E6" s="2">
-        <v>205</v>
+        <v>180</v>
       </c>
       <c r="F6" s="2">
         <v>205</v>
@@ -404,7 +415,7 @@
         <v>25</v>
       </c>
       <c r="F7" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="4:6" x14ac:dyDescent="0.3">
@@ -448,7 +459,7 @@
         <v>52</v>
       </c>
       <c r="F11" s="2">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="4:6" x14ac:dyDescent="0.3">
@@ -470,7 +481,7 @@
         <v>45</v>
       </c>
       <c r="F13" s="2">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="4:6" x14ac:dyDescent="0.3">
@@ -506,15 +517,25 @@
         <v>75</v>
       </c>
     </row>
-    <row r="17" spans="4:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D17" s="4">
         <v>46139</v>
       </c>
       <c r="E17" s="2">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F17" s="2">
-        <v>73</v>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="H19">
+        <f>SUM(E6:E17)</f>
+        <v>660</v>
+      </c>
+      <c r="I19">
+        <f>SUM(F6:F17)</f>
+        <v>1000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>